<commit_message>
Reset to remove Thinzar's dataset completely, then commit all future changes back.
</commit_message>
<xml_diff>
--- a/Tests/Validation/Canola/ObsPloschuk2021.xlsx
+++ b/Tests/Validation/Canola/ObsPloschuk2021.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilhuber\NextGen\ApsimX\Tests\Validation\Canola\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B7C8FA-AE9A-43F2-95BC-323A83DDBB69}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1133681F-7E4E-4BE1-88BF-0DD3CFD90A47}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10080" yWindow="2430" windowWidth="28800" windowHeight="13050" activeTab="4" xr2:uid="{03D29272-A8D3-49D2-9408-6969D9C41BBD}"/>
+    <workbookView xWindow="10080" yWindow="2430" windowWidth="28800" windowHeight="13050" activeTab="1" xr2:uid="{03D29272-A8D3-49D2-9408-6969D9C41BBD}"/>
   </bookViews>
   <sheets>
     <sheet name="Canola" sheetId="3" r:id="rId1"/>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">LAI_at_end_treatment!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">RUE_at_end_treatment!$A$1:$E$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">TimeSeries!$A$1:$G$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">TimeSeries!$A$1:$F$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="36">
   <si>
     <t>LAI</t>
   </si>
@@ -135,13 +135,7 @@
     <t>Canola.Aboveground.Wt</t>
   </si>
   <si>
-    <t>Canola.Grain.HarvestIndex</t>
-  </si>
-  <si>
     <t>Canola.Grain.HarvestIndexError</t>
-  </si>
-  <si>
-    <t>Canola.Leaf.CoverGreen</t>
   </si>
   <si>
     <t>Canola.Grain.Wt</t>
@@ -874,7 +868,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DCE79FF-CA68-45F5-80EF-0981CBC1EC45}">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
@@ -885,19 +879,18 @@
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.375" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22.875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.375" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="22.875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -911,10 +904,10 @@
         <v>14</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
         <v>7</v>
@@ -926,28 +919,25 @@
         <v>33</v>
       </c>
       <c r="J1" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="K1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O1" t="s">
-        <v>19</v>
-      </c>
-      <c r="P1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:15">
       <c r="A2" t="str">
         <f>"Exp_1_"&amp;D2</f>
         <v>Exp_1_Control</v>
@@ -974,31 +964,28 @@
         <v>7967.4337148168352</v>
       </c>
       <c r="I2">
-        <v>0.27700000000000002</v>
+        <v>1.0392304845413263E-2</v>
       </c>
       <c r="J2">
-        <v>1.0392304845413263E-2</v>
+        <v>11239</v>
       </c>
       <c r="K2">
-        <v>11239</v>
+        <v>277.12812921102034</v>
       </c>
       <c r="L2">
-        <v>277.12812921102034</v>
+        <v>15.7</v>
       </c>
       <c r="M2">
-        <v>15.7</v>
+        <v>1.0392304845413263</v>
       </c>
       <c r="N2">
-        <v>1.0392304845413263</v>
+        <v>3.7</v>
       </c>
       <c r="O2">
-        <v>3.7</v>
-      </c>
-      <c r="P2">
         <v>0.17320508075688773</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:15">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A7" si="0">"Exp_1_"&amp;D3</f>
         <v>Exp_1_Early_WL</v>
@@ -1025,31 +1012,28 @@
         <v>15761.662348876782</v>
       </c>
       <c r="I3">
-        <v>0.23899999999999999</v>
+        <v>1.9052558883257648E-2</v>
       </c>
       <c r="J3">
-        <v>1.9052558883257648E-2</v>
+        <v>9945</v>
       </c>
       <c r="K3">
-        <v>9945</v>
+        <v>162.81277591147446</v>
       </c>
       <c r="L3">
-        <v>162.81277591147446</v>
+        <v>14.3</v>
       </c>
       <c r="M3">
-        <v>14.3</v>
+        <v>2.9444863728670914</v>
       </c>
       <c r="N3">
-        <v>2.9444863728670914</v>
+        <v>3.7</v>
       </c>
       <c r="O3">
-        <v>3.7</v>
-      </c>
-      <c r="P3">
         <v>0.34641016151377546</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:15">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -1076,31 +1060,28 @@
         <v>5369.3575034635196</v>
       </c>
       <c r="I4">
-        <v>0.223</v>
+        <v>1.212435565298214E-2</v>
       </c>
       <c r="J4">
-        <v>1.212435565298214E-2</v>
+        <v>10828</v>
       </c>
       <c r="K4">
-        <v>10828</v>
+        <v>495.36653096469888</v>
       </c>
       <c r="L4">
-        <v>495.36653096469888</v>
+        <v>10.1</v>
       </c>
       <c r="M4">
-        <v>10.1</v>
+        <v>0.51961524227066314</v>
       </c>
       <c r="N4">
-        <v>0.51961524227066314</v>
+        <v>3.4</v>
       </c>
       <c r="O4">
-        <v>3.4</v>
-      </c>
-      <c r="P4">
         <v>0.17320508075688773</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:15">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -1127,31 +1108,28 @@
         <v>28059.223082615812</v>
       </c>
       <c r="I5">
-        <v>0.30499999999999999</v>
+        <v>1.0392304845413263E-2</v>
       </c>
       <c r="J5">
-        <v>1.0392304845413263E-2</v>
+        <v>13150</v>
       </c>
       <c r="K5">
-        <v>13150</v>
+        <v>3363.6426682987594</v>
       </c>
       <c r="L5">
-        <v>3363.6426682987594</v>
+        <v>13.3</v>
       </c>
       <c r="M5">
-        <v>13.3</v>
+        <v>0.8660254037844386</v>
       </c>
       <c r="N5">
-        <v>0.8660254037844386</v>
+        <v>3.7</v>
       </c>
       <c r="O5">
-        <v>3.7</v>
-      </c>
-      <c r="P5">
         <v>0.17320508075688773</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:15">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -1178,31 +1156,28 @@
         <v>19398.969044771424</v>
       </c>
       <c r="I6">
-        <v>0.30499999999999999</v>
+        <v>8.6602540378443865E-3</v>
       </c>
       <c r="J6">
-        <v>8.6602540378443865E-3</v>
+        <v>10457</v>
       </c>
       <c r="K6">
-        <v>10457</v>
+        <v>2346.9288442558286</v>
       </c>
       <c r="L6">
-        <v>2346.9288442558286</v>
+        <v>12.7</v>
       </c>
       <c r="M6">
-        <v>12.7</v>
+        <v>0.8660254037844386</v>
       </c>
       <c r="N6">
-        <v>0.8660254037844386</v>
+        <v>3.4</v>
       </c>
       <c r="O6">
-        <v>3.4</v>
-      </c>
-      <c r="P6">
         <v>0.17320508075688773</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:15">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -1229,27 +1204,24 @@
         <v>14202.816622064793</v>
       </c>
       <c r="I7">
-        <v>0.23899999999999999</v>
+        <v>2.5980762113533156E-2</v>
       </c>
       <c r="J7">
-        <v>2.5980762113533156E-2</v>
+        <v>6353</v>
       </c>
       <c r="K7">
-        <v>6353</v>
+        <v>1988.3943270890711</v>
       </c>
       <c r="L7">
-        <v>1988.3943270890711</v>
+        <v>9.4</v>
       </c>
       <c r="M7">
-        <v>9.4</v>
+        <v>0.69282032302755092</v>
       </c>
       <c r="N7">
-        <v>0.69282032302755092</v>
+        <v>3.2</v>
       </c>
       <c r="O7">
-        <v>3.2</v>
-      </c>
-      <c r="P7">
         <v>0.34641016151377546</v>
       </c>
     </row>
@@ -1510,6 +1482,7 @@
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1897,14 +1870,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CCDE50D-DC28-4398-95CA-92F7BC129FD5}">
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.75" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1921,13 +1894,10 @@
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:6">
       <c r="A2" t="str">
         <f>"Exp_1_"&amp;C2</f>
         <v>Exp_1_Control</v>
@@ -1944,11 +1914,8 @@
       <c r="E2" s="4">
         <v>42985</v>
       </c>
-      <c r="F2">
-        <v>0.57788944723618096</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A66" si="0">"Exp_1_"&amp;C3</f>
         <v>Exp_1_Control</v>
@@ -1966,11 +1933,8 @@
         <f>$E$2+D3</f>
         <v>42994</v>
       </c>
-      <c r="F3">
-        <v>0.91959798994974795</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -1988,11 +1952,8 @@
         <f t="shared" ref="E4:E9" si="1">$E$2+D4</f>
         <v>43018</v>
       </c>
-      <c r="F4">
-        <v>0.95477386934673303</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2010,11 +1971,8 @@
         <f t="shared" si="1"/>
         <v>43031</v>
       </c>
-      <c r="F5">
-        <v>0.96482412060301503</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2032,11 +1990,8 @@
         <f t="shared" si="1"/>
         <v>43034</v>
       </c>
-      <c r="F6">
-        <v>0.904522613065326</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2054,11 +2009,8 @@
         <f t="shared" si="1"/>
         <v>43042</v>
       </c>
-      <c r="F7">
-        <v>0.89447236180904399</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2076,11 +2028,8 @@
         <f t="shared" si="1"/>
         <v>43051</v>
       </c>
-      <c r="F8">
-        <v>0.82412060301507495</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2098,11 +2047,8 @@
         <f t="shared" si="1"/>
         <v>43056</v>
       </c>
-      <c r="F9">
-        <v>0.67839195979899403</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2120,11 +2066,8 @@
         <f>$E$2+D10</f>
         <v>42995</v>
       </c>
-      <c r="F10">
-        <v>0.56281407035175901</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2142,11 +2085,8 @@
         <f t="shared" ref="E11:E17" si="2">$E$2+D11</f>
         <v>43001</v>
       </c>
-      <c r="F11">
-        <v>0.41708542713567798</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2164,11 +2104,8 @@
         <f t="shared" si="2"/>
         <v>43018</v>
       </c>
-      <c r="F12">
-        <v>0.86934673366834103</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2186,11 +2123,8 @@
         <f t="shared" si="2"/>
         <v>43031</v>
       </c>
-      <c r="F13">
-        <v>0.80904522613065299</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2208,11 +2142,8 @@
         <f t="shared" si="2"/>
         <v>43035</v>
       </c>
-      <c r="F14">
-        <v>0.85929648241206003</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2230,11 +2161,8 @@
         <f t="shared" si="2"/>
         <v>43042</v>
       </c>
-      <c r="F15">
-        <v>0.81407035175879405</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2252,11 +2180,8 @@
         <f t="shared" si="2"/>
         <v>43051</v>
       </c>
-      <c r="F16">
-        <v>0.85929648241206003</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2274,11 +2199,8 @@
         <f t="shared" si="2"/>
         <v>43057</v>
       </c>
-      <c r="F17">
-        <v>0.80904522613065299</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2296,11 +2218,8 @@
         <f>$E$2+D18</f>
         <v>43017</v>
       </c>
-      <c r="F18">
-        <v>0.904522613065326</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2318,11 +2237,8 @@
         <f t="shared" ref="E19:E23" si="3">$E$2+D19</f>
         <v>43031</v>
       </c>
-      <c r="F19">
-        <v>0.51758793969849204</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2340,11 +2256,8 @@
         <f t="shared" si="3"/>
         <v>43035</v>
       </c>
-      <c r="F20">
-        <v>0.32663316582914498</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2362,11 +2275,8 @@
         <f t="shared" si="3"/>
         <v>43042</v>
       </c>
-      <c r="F21">
-        <v>0.33668341708542598</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2384,11 +2294,8 @@
         <f t="shared" si="3"/>
         <v>43052</v>
       </c>
-      <c r="F22">
-        <v>0.46733668341708501</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2406,11 +2313,8 @@
         <f t="shared" si="3"/>
         <v>43057</v>
       </c>
-      <c r="F23">
-        <v>0.34170854271356699</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
+    </row>
+    <row r="24" spans="1:5">
       <c r="A24" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2427,11 +2331,8 @@
       <c r="E24" s="4">
         <v>43361</v>
       </c>
-      <c r="F24">
-        <v>0.25974025974025999</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
+    </row>
+    <row r="25" spans="1:5">
       <c r="A25" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2449,11 +2350,8 @@
         <f>$E$24+D25</f>
         <v>43369</v>
       </c>
-      <c r="F25">
-        <v>0.74025974025973995</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
+    </row>
+    <row r="26" spans="1:5">
       <c r="A26" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2471,11 +2369,8 @@
         <f t="shared" ref="E26:E33" si="4">$E$24+D26</f>
         <v>43377</v>
       </c>
-      <c r="F26">
-        <v>0.92207792207792205</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
+    </row>
+    <row r="27" spans="1:5">
       <c r="A27" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2493,11 +2388,8 @@
         <f t="shared" si="4"/>
         <v>43380</v>
       </c>
-      <c r="F27">
-        <v>0.89610389610389596</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
+    </row>
+    <row r="28" spans="1:5">
       <c r="A28" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2515,11 +2407,8 @@
         <f t="shared" si="4"/>
         <v>43385</v>
       </c>
-      <c r="F28">
-        <v>0.92857142857142905</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
+    </row>
+    <row r="29" spans="1:5">
       <c r="A29" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2537,11 +2426,8 @@
         <f t="shared" si="4"/>
         <v>43391</v>
       </c>
-      <c r="F29">
-        <v>0.95454545454545503</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2559,11 +2445,8 @@
         <f t="shared" si="4"/>
         <v>43404</v>
       </c>
-      <c r="F30">
-        <v>0.84415584415584399</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
+    </row>
+    <row r="31" spans="1:5">
       <c r="A31" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2581,11 +2464,8 @@
         <f t="shared" si="4"/>
         <v>43413</v>
       </c>
-      <c r="F31">
-        <v>0.84415584415584399</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
+    </row>
+    <row r="32" spans="1:5">
       <c r="A32" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2603,11 +2483,8 @@
         <f t="shared" si="4"/>
         <v>43420</v>
       </c>
-      <c r="F32">
-        <v>0.84415584415584399</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2625,11 +2502,8 @@
         <f t="shared" si="4"/>
         <v>43426</v>
       </c>
-      <c r="F33">
-        <v>0.68181818181818199</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2647,11 +2521,8 @@
         <f>$E$24+D34</f>
         <v>43369</v>
       </c>
-      <c r="F34">
-        <v>0.73376623376623396</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
+    </row>
+    <row r="35" spans="1:6">
       <c r="A35" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2669,11 +2540,8 @@
         <f t="shared" ref="E35:E42" si="5">$E$24+D35</f>
         <v>43377</v>
       </c>
-      <c r="F35">
-        <v>8.4415584415585096E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2691,11 +2559,8 @@
         <f t="shared" si="5"/>
         <v>43380</v>
       </c>
-      <c r="F36">
-        <v>0.103896103896104</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2713,11 +2578,8 @@
         <f t="shared" si="5"/>
         <v>43385</v>
       </c>
-      <c r="F37">
-        <v>0.31818181818181801</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
+    </row>
+    <row r="38" spans="1:6">
       <c r="A38" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2735,11 +2597,8 @@
         <f t="shared" si="5"/>
         <v>43391</v>
       </c>
-      <c r="F38">
-        <v>0.415584415584416</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
+    </row>
+    <row r="39" spans="1:6">
       <c r="A39" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2757,11 +2616,8 @@
         <f t="shared" si="5"/>
         <v>43404</v>
       </c>
-      <c r="F39">
-        <v>0.53896103896103897</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+    </row>
+    <row r="40" spans="1:6">
       <c r="A40" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2779,11 +2635,8 @@
         <f t="shared" si="5"/>
         <v>43413</v>
       </c>
-      <c r="F40">
-        <v>0.61038961038961004</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
+    </row>
+    <row r="41" spans="1:6">
       <c r="A41" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2801,11 +2654,8 @@
         <f t="shared" si="5"/>
         <v>43420</v>
       </c>
-      <c r="F41">
-        <v>0.48051948051948101</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
+    </row>
+    <row r="42" spans="1:6">
       <c r="A42" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -2823,11 +2673,8 @@
         <f t="shared" si="5"/>
         <v>43426</v>
       </c>
-      <c r="F42">
-        <v>0.52597402597402598</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
+    </row>
+    <row r="43" spans="1:6">
       <c r="A43" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2845,11 +2692,8 @@
         <f>$E$24+D43</f>
         <v>43391</v>
       </c>
-      <c r="F43">
-        <v>0.75324675324675305</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
+    </row>
+    <row r="44" spans="1:6">
       <c r="A44" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2867,11 +2711,8 @@
         <f t="shared" ref="E44:E47" si="6">$E$24+D44</f>
         <v>43404</v>
       </c>
-      <c r="F44">
-        <v>0.29220779220779203</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
+    </row>
+    <row r="45" spans="1:6">
       <c r="A45" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2889,11 +2730,8 @@
         <f t="shared" si="6"/>
         <v>43413</v>
       </c>
-      <c r="F45">
-        <v>0.28571428571428598</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7">
+    </row>
+    <row r="46" spans="1:6">
       <c r="A46" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2911,11 +2749,8 @@
         <f t="shared" si="6"/>
         <v>43420</v>
       </c>
-      <c r="F46">
-        <v>0.31168831168831101</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
+    </row>
+    <row r="47" spans="1:6">
       <c r="A47" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -2933,11 +2768,8 @@
         <f t="shared" si="6"/>
         <v>43426</v>
       </c>
-      <c r="F47">
-        <v>0.25974025974025999</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7">
+    </row>
+    <row r="48" spans="1:6">
       <c r="A48" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2954,11 +2786,11 @@
       <c r="E48" s="4">
         <v>42985</v>
       </c>
-      <c r="G48">
+      <c r="F48">
         <v>44.198895027624502</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:6">
       <c r="A49" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2976,11 +2808,11 @@
         <f>$E$48+D49</f>
         <v>42999</v>
       </c>
-      <c r="G49">
+      <c r="F49">
         <v>176.79558011049801</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:6">
       <c r="A50" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -2998,11 +2830,11 @@
         <f t="shared" ref="E50:E57" si="7">$E$48+D50</f>
         <v>43014</v>
       </c>
-      <c r="G50">
+      <c r="F50">
         <v>574.58563535911696</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:6">
       <c r="A51" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -3020,11 +2852,11 @@
         <f t="shared" si="7"/>
         <v>43028</v>
       </c>
-      <c r="G51">
+      <c r="F51">
         <v>1060.7734806629801</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:6">
       <c r="A52" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -3042,11 +2874,11 @@
         <f t="shared" si="7"/>
         <v>43072</v>
       </c>
-      <c r="G52">
+      <c r="F52">
         <v>2651.93370165745</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:6">
       <c r="A53" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -3064,11 +2896,11 @@
         <f t="shared" si="7"/>
         <v>42999</v>
       </c>
-      <c r="G53">
+      <c r="F53">
         <v>88.397790055250795</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:6">
       <c r="A54" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -3086,11 +2918,11 @@
         <f t="shared" si="7"/>
         <v>43028</v>
       </c>
-      <c r="G54">
+      <c r="F54">
         <v>574.58563535911696</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:6">
       <c r="A55" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -3108,11 +2940,11 @@
         <f t="shared" si="7"/>
         <v>43072</v>
       </c>
-      <c r="G55">
+      <c r="F55">
         <v>2232.0441988950201</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:6">
       <c r="A56" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -3130,11 +2962,11 @@
         <f t="shared" si="7"/>
         <v>43028</v>
       </c>
-      <c r="G56">
+      <c r="F56">
         <v>928.17679558011105</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:6">
       <c r="A57" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -3152,11 +2984,11 @@
         <f t="shared" si="7"/>
         <v>43072</v>
       </c>
-      <c r="G57">
+      <c r="F57">
         <v>1745.8563535911601</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:6">
       <c r="A58" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -3173,11 +3005,11 @@
       <c r="E58" s="4">
         <v>43361</v>
       </c>
-      <c r="G58">
+      <c r="F58">
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:6">
       <c r="A59" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -3195,11 +3027,11 @@
         <f>$E$58+D59</f>
         <v>43375</v>
       </c>
-      <c r="G59">
+      <c r="F59">
         <v>309.39226519337302</v>
       </c>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:6">
       <c r="A60" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -3217,11 +3049,11 @@
         <f t="shared" ref="E60:E67" si="8">$E$58+D60</f>
         <v>43383</v>
       </c>
-      <c r="G60">
+      <c r="F60">
         <v>353.59116022099602</v>
       </c>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:6">
       <c r="A61" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -3239,11 +3071,11 @@
         <f t="shared" si="8"/>
         <v>43397</v>
       </c>
-      <c r="G61">
+      <c r="F61">
         <v>795.58011049723905</v>
       </c>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:6">
       <c r="A62" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Control</v>
@@ -3261,11 +3093,11 @@
         <f t="shared" si="8"/>
         <v>43440</v>
       </c>
-      <c r="G62">
+      <c r="F62">
         <v>2033.14917127071</v>
       </c>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:6">
       <c r="A63" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -3283,11 +3115,11 @@
         <f t="shared" si="8"/>
         <v>43375</v>
       </c>
-      <c r="G63">
+      <c r="F63">
         <v>132.59668508287501</v>
       </c>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:6">
       <c r="A64" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -3305,11 +3137,11 @@
         <f t="shared" si="8"/>
         <v>43397</v>
       </c>
-      <c r="G64">
+      <c r="F64">
         <v>176.79558011049801</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:6">
       <c r="A65" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Early_WL</v>
@@ -3327,11 +3159,11 @@
         <f t="shared" si="8"/>
         <v>43440</v>
       </c>
-      <c r="G65">
+      <c r="F65">
         <v>1480.6629834254099</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:6">
       <c r="A66" t="str">
         <f t="shared" si="0"/>
         <v>Exp_1_Late_WL</v>
@@ -3349,11 +3181,11 @@
         <f t="shared" si="8"/>
         <v>43397</v>
       </c>
-      <c r="G66">
+      <c r="F66">
         <v>596.685082872929</v>
       </c>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" spans="1:6">
       <c r="A67" t="str">
         <f t="shared" ref="A67" si="9">"Exp_1_"&amp;C67</f>
         <v>Exp_1_Late_WL</v>
@@ -3371,7 +3203,7 @@
         <f t="shared" si="8"/>
         <v>43440</v>
       </c>
-      <c r="G67">
+      <c r="F67">
         <v>795.58011049723905</v>
       </c>
     </row>

</xml_diff>